<commit_message>
Sync refined P006–P010 engineering XLSX and add missing P009 workbook
</commit_message>
<xml_diff>
--- a/papers/P006/P006_工程复现问题清单_v1.xlsx
+++ b/papers/P006/P006_工程复现问题清单_v1.xlsx
@@ -30,13 +30,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF122C45"/>
+        <fgColor rgb="FF182D49"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF0F5FA"/>
+        <fgColor rgb="FFF1F5F9"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -57,7 +57,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFill="1" applyFont="1" applyAlignment="1">
       <alignment wrapText="1" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
@@ -72,15 +72,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr defaultRowHeight="25"/>
   <cols>
-    <col min="1" max="1" width="25" customWidth="1"/>
-    <col min="2" max="2" width="52" customWidth="1"/>
-    <col min="3" max="3" width="94" customWidth="1"/>
+    <col min="1" max="1" width="27" customWidth="1"/>
+    <col min="2" max="2" width="53" customWidth="1"/>
+    <col min="3" max="3" width="98" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="35" customHeight="1">
+    <row r="1" ht="36" customHeight="1">
       <c r="A1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">主题</t>
@@ -97,7 +97,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="88" customHeight="1">
+    <row r="2" ht="87" customHeight="1">
       <c r="A2" t="inlineStr" s="0">
         <is>
           <t xml:space="preserve">起点与LLM底座</t>
@@ -114,7 +114,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="88" customHeight="1">
+    <row r="3" ht="78" customHeight="1">
       <c r="A3" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Bandit究竟是什么</t>
@@ -127,11 +127,11 @@
       </c>
       <c r="C3" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">它是选择“下轮挖因子 Factor”还是“改预测模型 Model”的Python统计调度器。名字来自双臂老虎机：每轮只能试一个方向，只能观察这个方向的实验结果，逐步学习如何分配研发机会；不是由LLM直接选方向。</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="124" customHeight="1">
+          <t xml:space="preserve">它是Python研发调度器：每轮只能选择挖因子Factor或改预测模型Model，试完才能看到所选方向的结果。名称来自“两臂老虎机”的边试边学问题；不是LLM自己决定研发方向。</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="109" customHeight="1">
       <c r="A4" t="inlineStr" s="0">
         <is>
           <t xml:space="preserve">Bandit怎样选择</t>
@@ -144,11 +144,11 @@
       </c>
       <c r="C4" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">算法是二臂Contextual Thompson Sampling：先看当前策略8个指标；Factor/Model各保存一套“预期效果+不确定程度”，分别随机抽一组可能的系数，与8个指标相乘求和，选择抽样分数更高的方向。证据不足的方向仍有探索机会。图解、数字例子与源码入口：https://github.com/epshoron/JXwork/blob/main/papers/P006/P006_BANDIT_COSTEER_GUIDE.md</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="88" customHeight="1">
+          <t xml:space="preserve">使用双臂Contextual Thompson Sampling：读取当前策略8个指标；Factor和Model各保存“预期效果+不确定性”，每轮各随机抽一组系数与指标加权求分，选择较高者。随机抽样让数据不足的方向仍有探索机会。数字例子与代码图解：https://github.com/epshoron/JXwork/blob/main/papers/P006/P006_BANDIT_COSTEER_GUIDE.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="78" customHeight="1">
       <c r="A5" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Bandit怎样学习</t>
@@ -161,11 +161,11 @@
       </c>
       <c r="C5" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">回测后程序只记录刚才做过的方向，并更新该方向的统计模型；另一方向本轮没有新证据。论文描述按动作效果更新，但当前bandit.py实际把8个回测指标加权成反馈分数，并非直接“新评分−旧评分”；下一轮再从两套概率模型重新抽样。</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="88" customHeight="1">
+          <t xml:space="preserve">实验后只更新**真正选择过的方向**的统计模型，另一条本轮没有新证据。论文概括为按动作效果反馈；当前bandit.py实际用8项指标的加权和作为奖励，并非直接“新分数−旧分数”。</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="78" customHeight="1">
       <c r="A6" t="inlineStr" s="0">
         <is>
           <t xml:space="preserve">谁提出研究假设</t>
@@ -178,11 +178,11 @@
       </c>
       <c r="C6" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">都由Synthesis阶段的LLM提出。选Factor时，LLM根据已有实验提出新金融信号假设；选Model时，LLM提出网络结构、层数或超参数改进。Bandit只决定做哪一类任务，本身既不发明因子，也不设计神经网络。</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="88" customHeight="1">
+          <t xml:space="preserve">由Synthesis的LLM提出：Bandit选Factor，LLM构思新因子；选Model，LLM提出预测模型架构/超参数改进。Bandit本身只选方向。</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="78" customHeight="1">
       <c r="A7" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Prompt与任务输出</t>
@@ -195,134 +195,117 @@
       </c>
       <c r="C7" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">程序把选定方向的说明、历史成败、当前优秀方案和输出规范装成Prompt。LLM先返回JSON研究假设；再转成开发任务：Factor描述公式和变量，Model描述架构与训练超参数。不是把原始行情表直接传给LLM，也不是一步直接得到可运行代码。</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="88" customHeight="1">
+          <t xml:space="preserve">程序按所选分支，把当前较优成果、历史实验/反馈、研究要求放进Prompt。LLM输出JSON研究假设，再转开发任务：Factor侧描述公式/变量，Model侧描述架构/训练参数。</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="87" customHeight="1">
       <c r="A8" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Co-STEER负责什么</t>
+          <t xml:space="preserve">Co-STEER执行与调度</t>
         </is>
       </c>
       <c r="B8" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Co-STEER到底是什么，内部怎样写代码和修复？</t>
+          <t xml:space="preserve">它究竟怎么把假设实现为可运行代码？DAG做什么？</t>
         </is>
       </c>
       <c r="C8" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">它是把研究方案变成可运行Python的代码开发引擎：检索以前类似任务→LLM写/改代码→真实执行与查错→根据反馈修复→保存经验。不是另一套Bandit；复杂任务还能按依赖分步骤处理。</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="88" customHeight="1">
+          <t xml:space="preserve">Co-STEER是代码开发引擎：先按DAG（任务先后依赖图）安排子任务，再检索类似代码、让LLM写/改Python、真实执行查错；失败会调整难度估计和执行顺序，修复经验供以后复用。它不负责选Factor/Model。</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="78" customHeight="1">
       <c r="A9" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Co-STEER任务排序</t>
+          <t xml:space="preserve">因子与模型怎样接力</t>
         </is>
       </c>
       <c r="B9" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">为什么要画DAG，它按什么顺序开发？</t>
+          <t xml:space="preserve">是两路同时跑，还是一轮只改一个？</t>
         </is>
       </c>
       <c r="C9" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">DAG是“谁必须先完成，下一步才能做什么”的任务关系图。Co-STEER先处理基础依赖，再做组合任务；若某步失败就提高其难度估计、重新安排顺序，而不是让LLM一次性乱写整个程序。</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="88" customHeight="1">
+          <t xml:space="preserve">每轮择一方向：新因子搭配当前较优预测模型测试，新模型使用当前较优因子集测试；评价成功再更新对应最佳版本。是轮流优化、共享结果，不是双线程始终并发。</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="87" customHeight="1">
       <c r="A10" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">因子与模型怎样接力</t>
+          <t xml:space="preserve">真实评价怎么做</t>
         </is>
       </c>
       <c r="B10" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">是两路同时跑，还是一轮只改一个？</t>
+          <t xml:space="preserve">因子能运行就算成功吗？怎样去重与比较？</t>
         </is>
       </c>
       <c r="C10" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">联合模式每轮由Bandit选Factor或Model之一；研究新因子时用当前较优预测模型测效果，研究新模型时用当前较优因子集合做输入。成功后更新相应的优秀版本，下一轮再选方向；这是交替协作，不等于两条线持续并行训练。</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="88" customHeight="1">
+          <t xml:space="preserve">不算。新因子先检查与已有优秀因子的相关性，论文使用相关性阈值0.99过滤近似重复，再和现有模型放进Qlib评价；新模型则用当前优秀因子集合训练回测。预测IC/ICIR及收益、回撤等真实指标决定评价，而非只让LLM自评分。</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="87" customHeight="1">
       <c r="A11" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">真实评价怎么做</t>
+          <t xml:space="preserve">因子库与池级增益</t>
         </is>
       </c>
       <c r="B11" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">因子能运行就算成功吗？怎样去重与比较？</t>
+          <t xml:space="preserve">这里的优秀因子库，和P005的因子池边际贡献一样吗？</t>
         </is>
       </c>
       <c r="C11" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">不算。新因子先检查与已有优秀因子的相关性，论文使用相关性阈值0.99过滤近似重复，再和现有模型放进Qlib评价；新模型则用当前优秀因子集合训练回测。预测IC/ICIR及收益、回撤等真实指标决定评价，而非只让LLM自评分。</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="88" customHeight="1">
+          <t xml:space="preserve">不完全一样。P006保存当前表现较好的因子和模型，尝试用新因子搭配现有模型改进效果；但未描述P005那种逐个新因子计算“加入前后整池加权分数差ΔΓ”的显式池级筛选，所以不能直接把两种“池”混为一谈。</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="78" customHeight="1">
       <c r="A12" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">因子库与池级增益</t>
+          <t xml:space="preserve">反馈与更新对象</t>
         </is>
       </c>
       <c r="B12" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">这里的优秀因子库，和P005的因子池边际贡献一样吗？</t>
+          <t xml:space="preserve">什么被保存和改进？Bandit或Co-STEER会训练LLM本身吗？</t>
         </is>
       </c>
       <c r="C12" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">不完全一样。P006保存当前表现较好的因子和模型，尝试用新因子搭配现有模型改进效果；但未描述P005那种逐个新因子计算“加入前后整池加权分数差ΔΓ”的显式池级筛选，所以不能直接把两种“池”混为一谈。</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="100" customHeight="1">
+          <t xml:space="preserve">Analysis把成败和解释反馈下一轮；Co-STEER积累代码修复经验；Bandit更新统计参数，Model侧训练下游预测器。没有证据显示研发用LLM本身做SFT/RL。</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="98" customHeight="1">
       <c r="A13" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">反馈与更新对象</t>
+          <t xml:space="preserve">源码和证据边界</t>
         </is>
       </c>
       <c r="B13" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">什么被保存和改进？Bandit或Co-STEER会训练LLM本身吗？</t>
+          <t xml:space="preserve">算法是原文真实写的，还是只看了简介？哪些能查源码？</t>
         </is>
       </c>
       <c r="C13" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Analysis将本轮表现、成功失败与原因反馈给下一轮Synthesis；Co-STEER另记代码修复经验。Bandit更新的是统计参数，Factor线更新候选和因子库，Model线可能训练下游预测模型；没有证据表明研发用LLM本身通过SFT/RL更新权重。</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="112" customHeight="1">
-      <c r="A14" t="inlineStr" s="0">
-        <is>
-          <t xml:space="preserve">源码和证据边界</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr" s="0">
-        <is>
-          <t xml:space="preserve">算法是原文真实写的，还是只看了简介？哪些能查源码？</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr" s="0">
-        <is>
           <t xml:space="preserve">论文§2与附录A.1/A.2给出Co-STEER和Bandit机制；公开RD-Agent仓库可以查到bandit.py、quant_proposal.py和CoSTEER源码。已核对原文与部分Python文件，但仓库持续更新，尚未运行完整复现或确定当前分支与论文提交版完全一致。详见：https://github.com/microsoft/RD-Agent</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C14"/>
+  <autoFilter ref="A1:C13"/>
   <hyperlinks>
-    <hyperlink ref="C4" r:id="rId1" tooltip="查看详细机制图解"/>
-    <hyperlink ref="C14" r:id="rId2" tooltip="查看详细机制图解"/>
+    <hyperlink ref="C4" r:id="rId1" tooltip="打开论文、源码或机制图解"/>
+    <hyperlink ref="C13" r:id="rId2" tooltip="打开论文、源码或机制图解"/>
   </hyperlinks>
 </worksheet>
 </file>
</xml_diff>